<commit_message>
Fix flash total size issue
</commit_message>
<xml_diff>
--- a/Projects/NUCLEO-H563ZI/Applications/ROT_S/OEMiROT.xlsx
+++ b/Projects/NUCLEO-H563ZI/Applications/ROT_S/OEMiROT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chens\STM32Cube\Repository\H5_V1.4.0\Projects\NUCLEO-H563ZI\Applications\ROT_S\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A217BA5-F840-44CE-9EA7-FEC8A630BE8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{058AD0AF-536E-4ECD-B389-BB69BEC6AC2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EA4F91E5-2F2C-41F9-ADC4-50A0D48CACE5}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EA4F91E5-2F2C-41F9-ADC4-50A0D48CACE5}"/>
   </bookViews>
   <sheets>
     <sheet name="OEMiROT + S only App" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="59">
   <si>
     <t>Flash area</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -274,6 +274,9 @@
   </si>
   <si>
     <t>S data size (nb pages)</t>
+  </si>
+  <si>
+    <t>total size  (KB)</t>
   </si>
 </sst>
 </file>
@@ -359,7 +362,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -370,6 +373,12 @@
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
@@ -409,12 +418,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -466,18 +476,18 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -490,8 +500,15 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="20% - Accent2" xfId="1" builtinId="34"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="6">
@@ -879,7 +896,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99923FCB-07F1-46D0-9A9C-FE8B055CF38C}">
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
@@ -1358,102 +1375,111 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
-      <c r="A17" s="12" t="s">
+    <row r="16" spans="1:11">
+      <c r="E16" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="F16" s="25">
+        <f>SUM(F7:F15)</f>
+        <v>504</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="B18" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="C18" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="D17" s="12" t="s">
+      <c r="D18" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="12" t="s">
+      <c r="E18" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="F17" s="12" t="s">
+      <c r="F18" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="G17" s="21"/>
-    </row>
-    <row r="18" spans="1:7">
-      <c r="A18" s="2" t="s">
+      <c r="G18" s="21"/>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B18" s="6" t="str">
+      <c r="B19" s="6" t="str">
         <f>E10</f>
         <v>C018000</v>
       </c>
-      <c r="C18" s="13" t="str">
-        <f>DEC2HEX(HEX2DEC(B18)+HEX2DEC(D18)-1)</f>
-        <v>C0183FF</v>
-      </c>
-      <c r="D18" s="14">
-        <v>400</v>
-      </c>
-      <c r="E18" s="14">
-        <f>HEX2DEC(D18)/$B$2/1024</f>
-        <v>0.125</v>
-      </c>
-      <c r="F18" s="4">
-        <f>HEX2DEC(D18)/1024</f>
-        <v>1</v>
-      </c>
-      <c r="G18" s="22"/>
-    </row>
-    <row r="19" spans="1:7">
-      <c r="A19" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B19" s="11" t="str">
-        <f>DEC2HEX(HEX2DEC(B18)+HEX2DEC(D18))</f>
-        <v>C018400</v>
-      </c>
       <c r="C19" s="13" t="str">
         <f>DEC2HEX(HEX2DEC(B19)+HEX2DEC(D19)-1)</f>
-        <v>C041BFF</v>
-      </c>
-      <c r="D19" s="14" t="str">
-        <f>DEC2HEX((F10)*1024-HEX2DEC(D18)-HEX2DEC(D20))</f>
-        <v>29800</v>
+        <v>C0183FF</v>
+      </c>
+      <c r="D19" s="14">
+        <v>400</v>
       </c>
       <c r="E19" s="14">
-        <f t="shared" ref="E19:E20" si="1">HEX2DEC(D19)/$B$2/1024</f>
-        <v>20.75</v>
+        <f>HEX2DEC(D19)/$B$2/1024</f>
+        <v>0.125</v>
       </c>
       <c r="F19" s="4">
-        <f t="shared" ref="F19:F20" si="2">HEX2DEC(D19)/1024</f>
-        <v>166</v>
+        <f>HEX2DEC(D19)/1024</f>
+        <v>1</v>
       </c>
       <c r="G19" s="22"/>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B20" s="11" t="str">
-        <f>DEC2HEX((HEX2DEC(B18)+F10*1024)-HEX2DEC(D20))</f>
-        <v>C041C00</v>
+        <f>DEC2HEX(HEX2DEC(B19)+HEX2DEC(D19))</f>
+        <v>C018400</v>
       </c>
       <c r="C20" s="13" t="str">
         <f>DEC2HEX(HEX2DEC(B20)+HEX2DEC(D20)-1)</f>
+        <v>C041BFF</v>
+      </c>
+      <c r="D20" s="14" t="str">
+        <f>DEC2HEX((F10)*1024-HEX2DEC(D19)-HEX2DEC(D21))</f>
+        <v>29800</v>
+      </c>
+      <c r="E20" s="14">
+        <f t="shared" ref="E20:E21" si="1">HEX2DEC(D20)/$B$2/1024</f>
+        <v>20.75</v>
+      </c>
+      <c r="F20" s="4">
+        <f t="shared" ref="F20:F21" si="2">HEX2DEC(D20)/1024</f>
+        <v>166</v>
+      </c>
+      <c r="G20" s="22"/>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21" s="11" t="str">
+        <f>DEC2HEX((HEX2DEC(B19)+F10*1024)-HEX2DEC(D21))</f>
+        <v>C041C00</v>
+      </c>
+      <c r="C21" s="13" t="str">
+        <f>DEC2HEX(HEX2DEC(B21)+HEX2DEC(D21)-1)</f>
         <v>C041FFF</v>
       </c>
-      <c r="D20" s="14">
+      <c r="D21" s="14">
         <v>400</v>
       </c>
-      <c r="E20" s="14">
+      <c r="E21" s="14">
         <f t="shared" si="1"/>
         <v>0.125</v>
       </c>
-      <c r="F20" s="4">
+      <c r="F21" s="4">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="G20" s="22"/>
+      <c r="G21" s="22"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -1480,8 +1506,8 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7 H10" xr:uid="{086C481C-D36E-437A-9AC5-9FB8DA1FBD4A}">
       <formula1>$I$1</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C19" xr:uid="{D6FA7859-AA3C-4242-A896-2F85780AF254}">
-      <formula1>B20</formula1>
+    <dataValidation type="whole" operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C20" xr:uid="{D6FA7859-AA3C-4242-A896-2F85780AF254}">
+      <formula1>B21</formula1>
     </dataValidation>
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F8:F9 F12:F15 F10:F11" xr:uid="{55A5B966-5FA6-4DAB-8198-D4659C47FBFA}">
       <formula1>0</formula1>

</xml_diff>

<commit_message>
Adjust flash layout for single slot case on 2MB H563 for CubeIDE project
</commit_message>
<xml_diff>
--- a/Projects/NUCLEO-H563ZI/Applications/ROT_S/OEMiROT.xlsx
+++ b/Projects/NUCLEO-H563ZI/Applications/ROT_S/OEMiROT.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chens\STM32Cube\Repository\H5_V1.4.0\Projects\NUCLEO-H563ZI\Applications\ROT_S\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{058AD0AF-536E-4ECD-B389-BB69BEC6AC2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F0E4925-ABD3-467A-A6DD-5E6CCF15D90D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EA4F91E5-2F2C-41F9-ADC4-50A0D48CACE5}"/>
   </bookViews>
   <sheets>
-    <sheet name="OEMiROT + S only App" sheetId="1" r:id="rId1"/>
+    <sheet name="OEMiROT + S only App (512KB)" sheetId="3" r:id="rId1"/>
+    <sheet name="OEMiROT + S only App (2MB)" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OEMiROT + S only App'!$A$6:$J$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'OEMiROT + S only App (2MB)'!$A$6:$J$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'OEMiROT + S only App (512KB)'!$A$6:$J$15</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,10 +43,28 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={13EC26EC-1EA7-4491-A58E-BEDC1F333067}</author>
+    <author>tc={C4BC7059-F8CF-4419-ADF2-26961ACEF965}</author>
   </authors>
   <commentList>
-    <comment ref="F6" authorId="0" shapeId="0" xr:uid="{13EC26EC-1EA7-4491-A58E-BEDC1F333067}">
+    <comment ref="F6" authorId="0" shapeId="0" xr:uid="{C4BC7059-F8CF-4419-ADF2-26961ACEF965}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Need to align to 8KB page size</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={38A4689F-4B1B-464D-979F-F9B810314B8B}</author>
+  </authors>
+  <commentList>
+    <comment ref="F6" authorId="0" shapeId="0" xr:uid="{38A4689F-4B1B-464D-979F-F9B810314B8B}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -57,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="59">
   <si>
     <t>Flash area</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -359,7 +379,7 @@
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -488,10 +508,10 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -511,7 +531,27 @@
     <cellStyle name="20% - Accent2" xfId="1" builtinId="34"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="10">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -554,6 +594,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -569,6 +619,16 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -888,14 +948,22 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="F6" dT="2025-03-10T03:53:56.17" personId="{DA7C2F05-062F-429C-8D88-B06321654FA0}" id="{13EC26EC-1EA7-4491-A58E-BEDC1F333067}">
+  <threadedComment ref="F6" dT="2025-03-10T03:53:56.17" personId="{DA7C2F05-062F-429C-8D88-B06321654FA0}" id="{C4BC7059-F8CF-4419-ADF2-26961ACEF965}">
+    <text>Need to align to 8KB page size</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="F6" dT="2025-03-10T03:53:56.17" personId="{DA7C2F05-062F-429C-8D88-B06321654FA0}" id="{38A4689F-4B1B-464D-979F-F9B810314B8B}">
     <text>Need to align to 8KB page size</text>
   </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99923FCB-07F1-46D0-9A9C-FE8B055CF38C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{795AC923-63B6-4460-BD12-9B91833135F5}">
   <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1164,7 +1232,7 @@
         <v>C018000</v>
       </c>
       <c r="F10" s="5">
-        <f>ROUNDDOWN((B1-F7-F8-F9-F15-F14-F13-F12)/16,0)*8</f>
+        <f>ROUNDDOWN((B1-F7-F8-F9-F15-F14-F13-F12)/16,0)*IF(H11="Yes",8,16)</f>
         <v>168</v>
       </c>
       <c r="G10" s="23" t="str">
@@ -1202,7 +1270,7 @@
         <v>C042000</v>
       </c>
       <c r="F11" s="5">
-        <f>F10</f>
+        <f>IF(H11="Yes",F10,0)</f>
         <v>168</v>
       </c>
       <c r="G11" s="23" t="str">
@@ -1249,7 +1317,7 @@
         <v>0</v>
       </c>
       <c r="H12" s="4" t="str">
-        <f>IF(UPPER($B$3)="YES", H9, 0)</f>
+        <f>IF(UPPER($B$3)="YES", H9, B4)</f>
         <v>No</v>
       </c>
       <c r="I12" s="4" t="s">
@@ -1482,45 +1550,682 @@
       <c r="G21" s="22"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="H7:K15">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+  <conditionalFormatting sqref="B3:B5">
+    <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B3:B5">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
-      <formula>"No"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+  <conditionalFormatting sqref="H7:K15">
+    <cfRule type="cellIs" dxfId="7" priority="3" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="8">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I7:K10 H11:K15 H8" xr:uid="{0AB68875-50C4-4C4A-899E-1034362D38A6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I7:K10 H11:K15 H8" xr:uid="{71462FC0-FF1C-4A72-B524-752C3DBCC95C}">
       <formula1>$I$1:$I$2</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F7" xr:uid="{F70CAB97-7C35-46A8-80C4-398CB2556795}">
+    <dataValidation type="whole" operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F7" xr:uid="{1CB1F42B-62C7-4A01-B6E6-92B9DEA63B1C}">
       <formula1>96</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7 H10" xr:uid="{086C481C-D36E-437A-9AC5-9FB8DA1FBD4A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7 H10" xr:uid="{24EB08C0-24DB-4CE7-A0B2-354EE95104C8}">
       <formula1>$I$1</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C20" xr:uid="{D6FA7859-AA3C-4242-A896-2F85780AF254}">
+    <dataValidation type="whole" operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C20" xr:uid="{8F42C9B6-09F1-4FD9-8BD4-9A816691AE23}">
       <formula1>B21</formula1>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F8:F9 F12:F15 F10:F11" xr:uid="{55A5B966-5FA6-4DAB-8198-D4659C47FBFA}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F8:F15" xr:uid="{9A4F1DA6-90CF-49D1-A1FA-CCCDBD00F75F}">
       <formula1>0</formula1>
       <formula2>512</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B5" xr:uid="{4BE1B0BC-FCD7-4C01-B98E-07DF4BF571E2}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B5" xr:uid="{C11A97BF-5436-4667-8437-D163CD315703}">
       <formula1>$H$1:$H$2</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H9" xr:uid="{E24C9E79-E2F6-4F3B-82E0-4F94A38438A4}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H9" xr:uid="{E279EABA-38C9-4B35-867D-BF877D72997D}">
       <formula1>$B$4</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E12 E13" xr:uid="{DC101747-246C-4190-8598-2286FB0E23DE}">
+    <dataValidation type="whole" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E12:E13" xr:uid="{D4B42958-159F-4CF2-A83D-130C225DE8FE}">
       <formula1>E13</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8C0673D-D5D7-48B6-A1D3-2697C5BD9CDD}">
+  <dimension ref="A1:K21"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="10">
+        <v>2048</v>
+      </c>
+      <c r="C1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" s="16" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="10">
+        <v>8</v>
+      </c>
+      <c r="H2" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="J2" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="16" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D4" s="10">
+        <v>1</v>
+      </c>
+      <c r="H4" s="16"/>
+      <c r="I4" s="16"/>
+      <c r="J4" s="16"/>
+      <c r="K4" s="16"/>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="16"/>
+      <c r="K5" s="16"/>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="I6" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="J6" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="K6" s="12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" s="1" customFormat="1">
+      <c r="A7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="7" t="str">
+        <f>D1</f>
+        <v>C000000</v>
+      </c>
+      <c r="F7" s="5">
+        <v>96</v>
+      </c>
+      <c r="G7" s="23" t="str">
+        <f>DEC2HEX(F7*1024)</f>
+        <v>18000</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="8" t="str">
+        <f>DEC2HEX(HEX2DEC(E7)+F7*1024)</f>
+        <v>C018000</v>
+      </c>
+      <c r="F8" s="4">
+        <f>IF(UPPER(H8)="YES", 8*$B$2, 0)</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="23" t="str">
+        <f t="shared" ref="G8:G15" si="0">DEC2HEX(F8*1024)</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="4" t="str">
+        <f>$B$5</f>
+        <v>No</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="E9" s="8" t="str">
+        <f>DEC2HEX(HEX2DEC(E8)+F8*1024)</f>
+        <v>C018000</v>
+      </c>
+      <c r="F9" s="4">
+        <f>IF(UPPER(H9)="YES", D4*$B$2, 0)</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="23" t="str">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H9" s="4" t="str">
+        <f>$B$4</f>
+        <v>No</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" s="1" customFormat="1">
+      <c r="A10" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="9" t="str">
+        <f>DEC2HEX(HEX2DEC(E9)+F9*1024)</f>
+        <v>C018000</v>
+      </c>
+      <c r="F10" s="5">
+        <f>ROUNDDOWN((B1-F7-F8-F9-F15-F14-F13-F12)/16,0)*IF(H11="Yes",8,16)</f>
+        <v>1872</v>
+      </c>
+      <c r="G10" s="23" t="str">
+        <f t="shared" si="0"/>
+        <v>1D4000</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" s="1" customFormat="1">
+      <c r="A11" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" s="9" t="str">
+        <f>DEC2HEX(HEX2DEC(E10)+F10*1024)</f>
+        <v>C1EC000</v>
+      </c>
+      <c r="F11" s="5">
+        <f>IF(H11="Yes",F10,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="23" t="str">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H11" s="5" t="str">
+        <f>B3</f>
+        <v>No</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="E12" s="8" t="str">
+        <f>DEC2HEX(HEX2DEC(E11)+F11*1024)</f>
+        <v>C1EC000</v>
+      </c>
+      <c r="F12" s="4">
+        <f>IF(UPPER(H12)="YES", D4*$F$9, 0)</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="23" t="str">
+        <f>DEC2HEX(F12*1024)</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="4" t="str">
+        <f>IF(UPPER($B$3)="YES", H9, B4)</f>
+        <v>No</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" s="8" t="str">
+        <f>DEC2HEX(HEX2DEC(E14)-F13*1024)</f>
+        <v>C1EE000</v>
+      </c>
+      <c r="F13" s="4">
+        <f>IF(UPPER(H13)="YES", 2*$B$2, 0)</f>
+        <v>16</v>
+      </c>
+      <c r="G13" s="23" t="str">
+        <f t="shared" si="0"/>
+        <v>4000</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" s="1" customFormat="1">
+      <c r="A14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="9" t="str">
+        <f>DEC2HEX(HEX2DEC(E15)-F14*1024)</f>
+        <v>C1F2000</v>
+      </c>
+      <c r="F14" s="5">
+        <v>48</v>
+      </c>
+      <c r="G14" s="23" t="str">
+        <f t="shared" si="0"/>
+        <v>C000</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="K14" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" s="1" customFormat="1">
+      <c r="A15" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E15" s="9" t="str">
+        <f>DEC2HEX((B1-F15)*1024 + HEX2DEC(D1))</f>
+        <v>C1FE000</v>
+      </c>
+      <c r="F15" s="5">
+        <f>1*B2</f>
+        <v>8</v>
+      </c>
+      <c r="G15" s="23" t="str">
+        <f t="shared" si="0"/>
+        <v>2000</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="J15" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="E16" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="F16" s="25">
+        <f>SUM(F7:F15)</f>
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="G18" s="21"/>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19" s="6" t="str">
+        <f>E10</f>
+        <v>C018000</v>
+      </c>
+      <c r="C19" s="13" t="str">
+        <f>DEC2HEX(HEX2DEC(B19)+HEX2DEC(D19)-1)</f>
+        <v>C0183FF</v>
+      </c>
+      <c r="D19" s="14">
+        <v>400</v>
+      </c>
+      <c r="E19" s="14">
+        <f>HEX2DEC(D19)/$B$2/1024</f>
+        <v>0.125</v>
+      </c>
+      <c r="F19" s="4">
+        <f>HEX2DEC(D19)/1024</f>
+        <v>1</v>
+      </c>
+      <c r="G19" s="22"/>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="11" t="str">
+        <f>DEC2HEX(HEX2DEC(B19)+HEX2DEC(D19))</f>
+        <v>C018400</v>
+      </c>
+      <c r="C20" s="13" t="str">
+        <f>DEC2HEX(HEX2DEC(B20)+HEX2DEC(D20)-1)</f>
+        <v>C1EBBFF</v>
+      </c>
+      <c r="D20" s="14" t="str">
+        <f>DEC2HEX((F10)*1024-HEX2DEC(D19)-HEX2DEC(D21))</f>
+        <v>1D3800</v>
+      </c>
+      <c r="E20" s="14">
+        <f t="shared" ref="E20:E21" si="1">HEX2DEC(D20)/$B$2/1024</f>
+        <v>233.75</v>
+      </c>
+      <c r="F20" s="4">
+        <f t="shared" ref="F20:F21" si="2">HEX2DEC(D20)/1024</f>
+        <v>1870</v>
+      </c>
+      <c r="G20" s="22"/>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21" s="11" t="str">
+        <f>DEC2HEX((HEX2DEC(B19)+F10*1024)-HEX2DEC(D21))</f>
+        <v>C1EBC00</v>
+      </c>
+      <c r="C21" s="13" t="str">
+        <f>DEC2HEX(HEX2DEC(B21)+HEX2DEC(D21)-1)</f>
+        <v>C1EBFFF</v>
+      </c>
+      <c r="D21" s="14">
+        <v>400</v>
+      </c>
+      <c r="E21" s="14">
+        <f t="shared" si="1"/>
+        <v>0.125</v>
+      </c>
+      <c r="F21" s="4">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="G21" s="22"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B3:B5">
+    <cfRule type="cellIs" dxfId="6" priority="2" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H7:K15">
+    <cfRule type="cellIs" dxfId="4" priority="4" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H7:H15">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="8">
+    <dataValidation type="whole" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E12:E13" xr:uid="{1E7D5FCD-EAE1-439B-B5C0-AFAE8C2DC84A}">
+      <formula1>E13</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H9" xr:uid="{BBF7D66F-5CE7-4792-B124-E95288622718}">
+      <formula1>$B$4</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B5" xr:uid="{8CE84D1A-343E-4C47-AA91-42473B0200F5}">
+      <formula1>$H$1:$H$2</formula1>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F8:F15" xr:uid="{29FD8F96-B79F-4710-BB27-E4E24603A23B}">
+      <formula1>0</formula1>
+      <formula2>512</formula2>
+    </dataValidation>
+    <dataValidation type="whole" operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C20" xr:uid="{8AFCBE6F-5E1B-43A9-9784-413A933B84BE}">
+      <formula1>B21</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7 H10" xr:uid="{CAEE0B3C-20E7-4412-B85F-732B8A63E9E5}">
+      <formula1>$I$1</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F7" xr:uid="{80C2949F-5D60-4B2B-8B6D-CD8B7A2552BC}">
+      <formula1>96</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I7:K10 H11:K15 H8" xr:uid="{BA070099-C40C-4C67-8D21-DF6C8567D0A8}">
+      <formula1>$I$1:$I$2</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update flash layout to remove EDATA slot
</commit_message>
<xml_diff>
--- a/Projects/NUCLEO-H563ZI/Applications/ROT_S/OEMiROT.xlsx
+++ b/Projects/NUCLEO-H563ZI/Applications/ROT_S/OEMiROT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chens\STM32Cube\Repository\H5_V1.4.0\Projects\NUCLEO-H563ZI\Applications\ROT_S\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F0E4925-ABD3-467A-A6DD-5E6CCF15D90D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFD5D420-BC87-426E-901B-EBB4FF6AD396}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EA4F91E5-2F2C-41F9-ADC4-50A0D48CACE5}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{EA4F91E5-2F2C-41F9-ADC4-50A0D48CACE5}"/>
   </bookViews>
   <sheets>
     <sheet name="OEMiROT + S only App (512KB)" sheetId="3" r:id="rId1"/>
@@ -1866,11 +1866,11 @@
       </c>
       <c r="F10" s="5">
         <f>ROUNDDOWN((B1-F7-F8-F9-F15-F14-F13-F12)/16,0)*IF(H11="Yes",8,16)</f>
-        <v>1872</v>
+        <v>1888</v>
       </c>
       <c r="G10" s="23" t="str">
         <f t="shared" si="0"/>
-        <v>1D4000</v>
+        <v>1D8000</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>5</v>
@@ -1900,7 +1900,7 @@
       </c>
       <c r="E11" s="9" t="str">
         <f>DEC2HEX(HEX2DEC(E10)+F10*1024)</f>
-        <v>C1EC000</v>
+        <v>C1F0000</v>
       </c>
       <c r="F11" s="5">
         <f>IF(H11="Yes",F10,0)</f>
@@ -1939,7 +1939,7 @@
       </c>
       <c r="E12" s="8" t="str">
         <f>DEC2HEX(HEX2DEC(E11)+F11*1024)</f>
-        <v>C1EC000</v>
+        <v>C1F0000</v>
       </c>
       <c r="F12" s="4">
         <f>IF(UPPER(H12)="YES", D4*$F$9, 0)</f>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="E13" s="8" t="str">
         <f>DEC2HEX(HEX2DEC(E14)-F13*1024)</f>
-        <v>C1EE000</v>
+        <v>C1F0000</v>
       </c>
       <c r="F13" s="4">
         <f>IF(UPPER(H13)="YES", 2*$B$2, 0)</f>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="E14" s="9" t="str">
         <f>DEC2HEX(HEX2DEC(E15)-F14*1024)</f>
-        <v>C1F2000</v>
+        <v>C1F4000</v>
       </c>
       <c r="F14" s="5">
         <v>48</v>
@@ -2053,18 +2053,18 @@
       </c>
       <c r="E15" s="9" t="str">
         <f>DEC2HEX((B1-F15)*1024 + HEX2DEC(D1))</f>
-        <v>C1FE000</v>
+        <v>C200000</v>
       </c>
       <c r="F15" s="5">
-        <f>1*B2</f>
-        <v>8</v>
+        <f>IF(H15="Yes",1*B2,0)</f>
+        <v>0</v>
       </c>
       <c r="G15" s="23" t="str">
         <f t="shared" si="0"/>
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I15" s="5" t="s">
         <v>6</v>
@@ -2082,7 +2082,7 @@
       </c>
       <c r="F16" s="25">
         <f>SUM(F7:F15)</f>
-        <v>2040</v>
+        <v>2048</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -2141,19 +2141,19 @@
       </c>
       <c r="C20" s="13" t="str">
         <f>DEC2HEX(HEX2DEC(B20)+HEX2DEC(D20)-1)</f>
-        <v>C1EBBFF</v>
+        <v>C1EFBFF</v>
       </c>
       <c r="D20" s="14" t="str">
         <f>DEC2HEX((F10)*1024-HEX2DEC(D19)-HEX2DEC(D21))</f>
-        <v>1D3800</v>
+        <v>1D7800</v>
       </c>
       <c r="E20" s="14">
         <f t="shared" ref="E20:E21" si="1">HEX2DEC(D20)/$B$2/1024</f>
-        <v>233.75</v>
+        <v>235.75</v>
       </c>
       <c r="F20" s="4">
         <f t="shared" ref="F20:F21" si="2">HEX2DEC(D20)/1024</f>
-        <v>1870</v>
+        <v>1886</v>
       </c>
       <c r="G20" s="22"/>
     </row>
@@ -2163,11 +2163,11 @@
       </c>
       <c r="B21" s="11" t="str">
         <f>DEC2HEX((HEX2DEC(B19)+F10*1024)-HEX2DEC(D21))</f>
-        <v>C1EBC00</v>
+        <v>C1EFC00</v>
       </c>
       <c r="C21" s="13" t="str">
         <f>DEC2HEX(HEX2DEC(B21)+HEX2DEC(D21)-1)</f>
-        <v>C1EBFFF</v>
+        <v>C1EFFFF</v>
       </c>
       <c r="D21" s="14">
         <v>400</v>

</xml_diff>